<commit_message>
site favicon + fresh data
</commit_message>
<xml_diff>
--- a/Grafik_CCEE_SLIVEN1_22_07_2026.xlsx
+++ b/Grafik_CCEE_SLIVEN1_22_07_2026.xlsx
@@ -1651,8 +1651,10 @@
       <c r="B50" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C50" s="11" t="n">
-        <v>0</v>
+      <c r="C50" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D50" s="5" t="n">
         <v>0</v>
@@ -1671,8 +1673,10 @@
       <c r="B51" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C51" s="11" t="n">
-        <v>0</v>
+      <c r="C51" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D51" s="5" t="n">
         <v>0</v>
@@ -1691,8 +1695,10 @@
       <c r="B52" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C52" s="11" t="n">
-        <v>0</v>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D52" s="5" t="n">
         <v>0</v>
@@ -1711,8 +1717,10 @@
       <c r="B53" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C53" s="11" t="n">
-        <v>0</v>
+      <c r="C53" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D53" s="5" t="n">
         <v>0</v>
@@ -1971,10 +1979,8 @@
       <c r="B66" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C66" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C66" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D66" s="5" t="n">
         <v>0</v>
@@ -1993,10 +1999,8 @@
       <c r="B67" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C67" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C67" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D67" s="5" t="n">
         <v>0</v>
@@ -2015,10 +2019,8 @@
       <c r="B68" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C68" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C68" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D68" s="5" t="n">
         <v>0</v>
@@ -2037,10 +2039,8 @@
       <c r="B69" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C69" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C69" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D69" s="5" t="n">
         <v>0</v>
@@ -2389,13 +2389,11 @@
       <c r="B85" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C85" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C85" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D85" s="5" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="E85" s="9">
         <f>IFERROR(MIN(1800,MAX(0,ROUND(C85+D85,0))),MIN(1800,MAX(0,D85)))</f>
@@ -2411,13 +2409,11 @@
       <c r="B86" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C86" s="10" t="inlineStr">
-        <is>
-          <t>Put Adex Solcast value here</t>
-        </is>
+      <c r="C86" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="D86" s="5" t="n">
-        <v>0</v>
+        <v>1800</v>
       </c>
       <c r="E86" s="9">
         <f>IFERROR(MIN(1800,MAX(0,ROUND(C86+D86,0))),MIN(1800,MAX(0,D86)))</f>
@@ -2593,11 +2589,13 @@
       <c r="B95" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C95" s="11" t="n">
-        <v>0</v>
+      <c r="C95" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D95" s="5" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="E95" s="9">
         <f>IFERROR(MIN(1800,MAX(0,ROUND(C95+D95,0))),MIN(1800,MAX(0,D95)))</f>
@@ -2613,11 +2611,13 @@
       <c r="B96" s="1" t="n">
         <v>46225</v>
       </c>
-      <c r="C96" s="11" t="n">
-        <v>0</v>
+      <c r="C96" s="10" t="inlineStr">
+        <is>
+          <t>Put Adex Solcast value here</t>
+        </is>
       </c>
       <c r="D96" s="5" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="E96" s="9">
         <f>IFERROR(MIN(1800,MAX(0,ROUND(C96+D96,0))),MIN(1800,MAX(0,D96)))</f>

</xml_diff>